<commit_message>
docs: update dummy test dataset (Dados_teste.xlsx)
</commit_message>
<xml_diff>
--- a/Dados_teste.xlsx
+++ b/Dados_teste.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3f5f01c5dd7b5426/Desktop/PROJETO/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projeto\Nova pasta\automatsuo_v3\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="8_{8562A23D-76C3-4E8C-8E74-0EC5F0539D32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EAFC4569-997F-42C0-9169-B46C609D7F82}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85AA74BC-75DF-4CF6-92F5-AB3209D933B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{117B8215-3417-4623-A5BD-AE40F1FA7C8F}"/>
+    <workbookView xWindow="3120" yWindow="3120" windowWidth="21600" windowHeight="11295" xr2:uid="{117B8215-3417-4623-A5BD-AE40F1FA7C8F}"/>
   </bookViews>
   <sheets>
     <sheet name="excelb" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="622" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="622" uniqueCount="143">
   <si>
     <t/>
   </si>
@@ -390,9 +390,6 @@
     <t>A003KB</t>
   </si>
   <si>
-    <t>A005KB</t>
-  </si>
-  <si>
     <t>A007KB</t>
   </si>
   <si>
@@ -402,9 +399,6 @@
     <t>A011KB</t>
   </si>
   <si>
-    <t>A013KB</t>
-  </si>
-  <si>
     <t>A015KB</t>
   </si>
   <si>
@@ -420,9 +414,6 @@
     <t>A023KB</t>
   </si>
   <si>
-    <t>A025KB</t>
-  </si>
-  <si>
     <t>A027KB</t>
   </si>
   <si>
@@ -438,21 +429,12 @@
     <t>A035KB</t>
   </si>
   <si>
-    <t>A037KB</t>
-  </si>
-  <si>
     <t>A039KB</t>
   </si>
   <si>
-    <t>A041KB</t>
-  </si>
-  <si>
     <t>A043KB</t>
   </si>
   <si>
-    <t>A045KB</t>
-  </si>
-  <si>
     <t>A047KB</t>
   </si>
   <si>
@@ -463,9 +445,6 @@
   </si>
   <si>
     <t>A053KB</t>
-  </si>
-  <si>
-    <t>A055KB</t>
   </si>
   <si>
     <t>A057KB</t>
@@ -970,7 +949,7 @@
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="1" t="s">
-        <v>149</v>
+        <v>142</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>0</v>
@@ -1198,7 +1177,7 @@
     </row>
     <row r="13" spans="1:8">
       <c r="A13" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>113</v>
@@ -1250,7 +1229,7 @@
     </row>
     <row r="15" spans="1:8">
       <c r="A15" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>113</v>
@@ -1302,7 +1281,7 @@
     </row>
     <row r="17" spans="1:8">
       <c r="A17" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>113</v>
@@ -1354,7 +1333,7 @@
     </row>
     <row r="19" spans="1:8">
       <c r="A19" s="2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>113</v>
@@ -1406,7 +1385,7 @@
     </row>
     <row r="21" spans="1:8">
       <c r="A21" s="2" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>113</v>
@@ -1458,7 +1437,7 @@
     </row>
     <row r="23" spans="1:8">
       <c r="A23" s="2" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>113</v>
@@ -1510,7 +1489,7 @@
     </row>
     <row r="25" spans="1:8">
       <c r="A25" s="2" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>113</v>
@@ -1562,7 +1541,7 @@
     </row>
     <row r="27" spans="1:8">
       <c r="A27" s="2" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>113</v>
@@ -1614,7 +1593,7 @@
     </row>
     <row r="29" spans="1:8">
       <c r="A29" s="2" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>113</v>
@@ -1666,7 +1645,7 @@
     </row>
     <row r="31" spans="1:8">
       <c r="A31" s="2" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>113</v>
@@ -1718,7 +1697,7 @@
     </row>
     <row r="33" spans="1:8">
       <c r="A33" s="2" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>113</v>
@@ -1770,7 +1749,7 @@
     </row>
     <row r="35" spans="1:8">
       <c r="A35" s="2" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>113</v>
@@ -1822,7 +1801,7 @@
     </row>
     <row r="37" spans="1:8">
       <c r="A37" s="2" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>113</v>
@@ -1874,7 +1853,7 @@
     </row>
     <row r="39" spans="1:8">
       <c r="A39" s="2" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>113</v>
@@ -1926,7 +1905,7 @@
     </row>
     <row r="41" spans="1:8">
       <c r="A41" s="2" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>113</v>
@@ -1978,7 +1957,7 @@
     </row>
     <row r="43" spans="1:8">
       <c r="A43" s="2" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>113</v>
@@ -2030,7 +2009,7 @@
     </row>
     <row r="45" spans="1:8">
       <c r="A45" s="2" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>113</v>
@@ -2082,7 +2061,7 @@
     </row>
     <row r="47" spans="1:8">
       <c r="A47" s="2" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>113</v>
@@ -2134,7 +2113,7 @@
     </row>
     <row r="49" spans="1:8">
       <c r="A49" s="2" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="B49" s="1" t="s">
         <v>113</v>
@@ -2186,7 +2165,7 @@
     </row>
     <row r="51" spans="1:8">
       <c r="A51" s="2" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="B51" s="1" t="s">
         <v>113</v>
@@ -2238,7 +2217,7 @@
     </row>
     <row r="53" spans="1:8">
       <c r="A53" s="2" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="B53" s="1" t="s">
         <v>113</v>
@@ -2290,7 +2269,7 @@
     </row>
     <row r="55" spans="1:8">
       <c r="A55" s="2" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="B55" s="1" t="s">
         <v>113</v>
@@ -2342,7 +2321,7 @@
     </row>
     <row r="57" spans="1:8">
       <c r="A57" s="2" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="B57" s="1" t="s">
         <v>113</v>
@@ -2394,7 +2373,7 @@
     </row>
     <row r="59" spans="1:8">
       <c r="A59" s="2" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="B59" s="1" t="s">
         <v>113</v>
@@ -2446,7 +2425,7 @@
     </row>
     <row r="61" spans="1:8">
       <c r="A61" s="2" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="B61" s="1" t="s">
         <v>113</v>
@@ -2498,7 +2477,7 @@
     </row>
     <row r="63" spans="1:8">
       <c r="A63" s="2" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="B63" s="1" t="s">
         <v>113</v>
@@ -2550,7 +2529,7 @@
     </row>
     <row r="65" spans="1:8">
       <c r="A65" s="2" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="B65" s="1" t="s">
         <v>113</v>
@@ -2602,7 +2581,7 @@
     </row>
     <row r="67" spans="1:8">
       <c r="A67" s="2" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="B67" s="1" t="s">
         <v>113</v>
@@ -2654,7 +2633,7 @@
     </row>
     <row r="69" spans="1:8">
       <c r="A69" s="2" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="B69" s="1" t="s">
         <v>113</v>
@@ -2706,7 +2685,7 @@
     </row>
     <row r="71" spans="1:8">
       <c r="A71" s="2" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="B71" s="1" t="s">
         <v>113</v>
@@ -2758,7 +2737,7 @@
     </row>
     <row r="73" spans="1:8">
       <c r="A73" s="2" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="B73" s="1" t="s">
         <v>113</v>
@@ -2810,7 +2789,7 @@
     </row>
     <row r="75" spans="1:8">
       <c r="A75" s="2" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="B75" s="1" t="s">
         <v>113</v>
@@ -2862,7 +2841,7 @@
     </row>
     <row r="77" spans="1:8">
       <c r="A77" s="2" t="s">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="B77" s="1" t="s">
         <v>113</v>

</xml_diff>